<commit_message>
fixed wdid name error
</commit_message>
<xml_diff>
--- a/data/structures.xlsx
+++ b/data/structures.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nickpenzel/github/transbasin_div/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{251DEA9F-A948-3441-AC36-B777B6AA1DE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A19A734D-B099-E64D-AF33-16A3DAF8FCA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24620" yWindow="-980" windowWidth="18900" windowHeight="17440" xr2:uid="{7D27D89D-4B56-384A-A3AD-4C7DA9952BD7}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17900" xr2:uid="{7D27D89D-4B56-384A-A3AD-4C7DA9952BD7}"/>
   </bookViews>
   <sheets>
     <sheet name="structures" sheetId="1" r:id="rId1"/>
@@ -332,9 +332,6 @@
     <t>7600572</t>
   </si>
   <si>
-    <t>wdid_telem</t>
-  </si>
-  <si>
     <t>4800572</t>
   </si>
   <si>
@@ -486,6 +483,9 @@
   </si>
   <si>
     <t>Stillwater Ditch</t>
+  </si>
+  <si>
+    <t>wdid</t>
   </si>
 </sst>
 </file>
@@ -917,13 +917,13 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>97</v>
+        <v>148</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D1" t="s">
         <v>0</v>
@@ -938,7 +938,7 @@
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I1" t="s">
         <v>4</v>
@@ -946,14 +946,14 @@
     </row>
     <row r="2" spans="1:11" ht="18" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>96</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -972,7 +972,7 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>66</v>
@@ -993,13 +993,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D4" t="s">
         <v>55</v>
@@ -1016,13 +1016,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>137</v>
       </c>
       <c r="D5" t="s">
         <v>56</v>
@@ -1037,10 +1037,10 @@
         <v>42</v>
       </c>
       <c r="H5" t="s">
+        <v>104</v>
+      </c>
+      <c r="I5" t="s">
         <v>105</v>
-      </c>
-      <c r="I5" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
@@ -1065,7 +1065,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>93</v>
@@ -1094,7 +1094,7 @@
         <v>7600600</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D8" t="s">
         <v>53</v>
@@ -1154,12 +1154,12 @@
         <v>8</v>
       </c>
       <c r="H10" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>70</v>
@@ -1180,7 +1180,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>71</v>
@@ -1199,7 +1199,7 @@
         <v>8</v>
       </c>
       <c r="H12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
@@ -1207,10 +1207,10 @@
         <v>5104603</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
         <v>10</v>
@@ -1225,12 +1225,12 @@
         <v>25</v>
       </c>
       <c r="I13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>92</v>
@@ -1257,7 +1257,7 @@
         <v>3604626</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -1274,7 +1274,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>88</v>
@@ -1297,7 +1297,7 @@
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>89</v>
@@ -1315,7 +1315,7 @@
         <v>8</v>
       </c>
       <c r="H17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
@@ -1326,7 +1326,7 @@
         <v>76</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1358,7 +1358,7 @@
         <v>8</v>
       </c>
       <c r="I19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
@@ -1369,7 +1369,7 @@
         <v>90</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
         <v>16</v>
@@ -1430,7 +1430,7 @@
     </row>
     <row r="23" spans="1:18" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B23" s="6">
         <v>1100501</v>
@@ -1449,7 +1449,7 @@
         <v>8</v>
       </c>
       <c r="H23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I23" t="s">
         <v>78</v>
@@ -1537,7 +1537,7 @@
         <v>8</v>
       </c>
       <c r="H27" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I27" t="s">
         <v>64</v>
@@ -1566,7 +1566,7 @@
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B29" s="6">
         <v>7900851</v>
@@ -1651,7 +1651,7 @@
         <v>82</v>
       </c>
       <c r="D33" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E33" t="s">
         <v>35</v>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="C34" s="6"/>
       <c r="D34" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E34" t="s">
         <v>35</v>
@@ -1710,7 +1710,7 @@
         <v>7804670</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D36" t="s">
         <v>39</v>
@@ -1727,7 +1727,7 @@
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>83</v>
@@ -1747,7 +1747,7 @@
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>84</v>
@@ -1785,7 +1785,7 @@
         <v>42</v>
       </c>
       <c r="H39" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="O39" s="3"/>
     </row>
@@ -1832,7 +1832,7 @@
         <v>42</v>
       </c>
       <c r="I41" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.2">
@@ -1843,7 +1843,7 @@
         <v>7100618</v>
       </c>
       <c r="D42" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E42" t="s">
         <v>46</v>
@@ -1863,10 +1863,10 @@
         <v>3204675</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D43" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E43" t="s">
         <v>46</v>
@@ -1911,7 +1911,7 @@
       </c>
       <c r="C45" s="6"/>
       <c r="D45" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E45" t="s">
         <v>46</v>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C46" s="6"/>
       <c r="D46" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E46" t="s">
         <v>35</v>
@@ -1949,13 +1949,13 @@
         <v>3004661</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C47" s="6">
         <v>6804659</v>
       </c>
       <c r="D47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E47" t="s">
         <v>35</v>
@@ -1975,7 +1975,7 @@
         <v>6000669</v>
       </c>
       <c r="D48" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E48" t="s">
         <v>46</v>
@@ -2035,7 +2035,7 @@
         <v>5804630</v>
       </c>
       <c r="D51" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E51" t="s">
         <v>50</v>
@@ -2055,7 +2055,7 @@
         <v>5804686</v>
       </c>
       <c r="D52" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E52" t="s">
         <v>50</v>

</xml_diff>